<commit_message>
keep spotting unique id
</commit_message>
<xml_diff>
--- a/data/processed/net_positions_by_activity.xlsx
+++ b/data/processed/net_positions_by_activity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATapia\IESE Dropbox\Alberto Tapia\IESE\Duro\ETS_repo\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA016618-381E-4E67-A80A-7B5322FB9BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCABF9A4-2197-4D4F-873B-C02A4CB60EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-8655" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -538,6 +538,10 @@
   <cols>
     <col min="1" max="1" width="9.36328125" customWidth="1"/>
     <col min="2" max="2" width="50.81640625" customWidth="1"/>
+    <col min="3" max="3" width="7.08984375" customWidth="1"/>
+    <col min="4" max="4" width="6.453125" customWidth="1"/>
+    <col min="5" max="5" width="6.7265625" customWidth="1"/>
+    <col min="6" max="6" width="6.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.35">
@@ -2898,6 +2902,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T38" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>